<commit_message>
Actualización automática de tasas-transfi.xlsx
</commit_message>
<xml_diff>
--- a/tasas-transfi.xlsx
+++ b/tasas-transfi.xlsx
@@ -724,8 +724,8 @@
           <t>Conversión del día 💰
 ✅ Dólar paralelo: 68
 Binance
-✅ 1000 Bs = 1.63 = 6071.0 pesos
-✅ 6071.0 pesos = 1.63 = 955.74 Bs
+✅ 1000 Bs = 1.61 = 5979.69 pesos
+✅ 5979.69 pesos = 1.6 = 933.9 Bs
 Promedio competencia
 ✅ Tasa pesos: 20
 ✅ Tasa Bs: 20
@@ -1142,10 +1142,10 @@
         <v/>
       </c>
       <c r="N10" s="8" t="n">
-        <v>612.42</v>
+        <v>619.8</v>
       </c>
       <c r="O10" s="8" t="n">
-        <v>3718</v>
+        <v>3706.21</v>
       </c>
     </row>
     <row r="11">
@@ -1178,10 +1178,10 @@
         <v/>
       </c>
       <c r="N12" s="8" t="n">
-        <v>3729.99</v>
+        <v>3739.32</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>587.2</v>
+        <v>584</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="42" thickBot="1">

</xml_diff>